<commit_message>
Daily MPR update | 11-02-26
</commit_message>
<xml_diff>
--- a/MPR/Role wise/Software Developer/Feb'26/MPR-Feb'26.xlsx
+++ b/MPR/Role wise/Software Developer/Feb'26/MPR-Feb'26.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\TH-PROJECT-NOTEBOOK\MPR\Role wise\Software Developer\Feb'26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D933697-BBC5-46A5-8727-2BD57D3A1C33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F07AF6-7E6E-4B71-AF78-3605D9611998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="29">
   <si>
     <t>SR#</t>
   </si>
@@ -85,6 +85,42 @@
   </si>
   <si>
     <t>Validation setup and hardening of TMS pending.</t>
+  </si>
+  <si>
+    <t>Staging Server Setup</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Analysis of Suksham Udhyam Sakhi App, Enterprise forms and identification of fields currently leaking from API</t>
+  </si>
+  <si>
+    <t>Suksham Udhyam Sakhi App</t>
+  </si>
+  <si>
+    <t>Received Internal Security Audit report of TMS, now working on fixing vulnerabilities</t>
+  </si>
+  <si>
+    <t>Switched to setup for Staging server provided by the Department for Hosting and security audit,                                  (1) Setup of Backend - Django (python) connected to localhost Test DB                                                                     (2) Exposing APIs for Auth and TMS</t>
+  </si>
+  <si>
+    <t>All other project development on hold, as staging server setup on priority</t>
+  </si>
+  <si>
+    <t>TMS</t>
+  </si>
+  <si>
+    <t>Switched to setup for Staging server provided by the Department for Hosting and security audit,                                  (1) Hosting TMS frontend on new server and setting up environment variables</t>
+  </si>
+  <si>
+    <t>Switched to setup for Staging server provided by the Department for Hosting and security audit,                                  (1) Locking Hosts for audit ready API and enforcing key based API protection.</t>
+  </si>
+  <si>
+    <t>Switched to setup for Staging server provided by the Department for Hosting and security audit,                                  (1) Fixed filter headers for batch list module in TMS                                               (2) Added object layer protections for restricted access aside from frontend</t>
+  </si>
+  <si>
+    <t>Switched to setup for Staging server provided by the Department for Hosting and security audit,                                  (1) Created and linked tables for audit and logging of different API requests being hit from different IP addresses</t>
   </si>
 </sst>
 </file>
@@ -135,7 +171,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -158,48 +194,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -216,14 +215,35 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -505,14 +525,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6806E486-C456-4888-BB52-4614915FD5B3}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6" style="10" customWidth="1"/>
+    <col min="2" max="2" width="34" style="10" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="10" customWidth="1"/>
+    <col min="4" max="5" width="14.5703125" style="10" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.28515625" style="10" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -542,16 +564,16 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
-      <c r="G2" s="8"/>
-    </row>
-    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -570,7 +592,7 @@
       <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>16</v>
       </c>
     </row>
@@ -578,16 +600,16 @@
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
-      <c r="G4" s="8"/>
-    </row>
-    <row r="5" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -606,11 +628,11 @@
       <c r="F5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="135" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -621,7 +643,7 @@
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E6" s="5">
         <v>46065</v>
@@ -629,14 +651,375 @@
       <c r="F6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="4" t="s">
         <v>15</v>
       </c>
     </row>
+    <row r="7" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="14">
+        <v>46065</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="14">
+        <v>46065</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="14">
+        <v>46065</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="14">
+        <v>46065</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="14">
+        <v>46065</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="14">
+        <v>46064</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" s="12"/>
+    </row>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" s="12"/>
+    </row>
+    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" s="12"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+    </row>
+    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" s="12"/>
+    </row>
+    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G18" s="12"/>
+    </row>
+    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" s="12"/>
+    </row>
+    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" s="12"/>
+    </row>
+    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G21" s="12"/>
+    </row>
+    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="12"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="12"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="12"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G24" s="12"/>
+    </row>
+    <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="12"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" s="12"/>
+    </row>
+    <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="12"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G26" s="12"/>
+    </row>
+    <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="12"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G27" s="12"/>
+    </row>
+    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="12"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="12"/>
+    </row>
+    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="12"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G29" s="12"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B23:G23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Change Request | 19-02-2026
</commit_message>
<xml_diff>
--- a/MPR/Role wise/Software Developer/Feb'26/MPR-Feb'26.xlsx
+++ b/MPR/Role wise/Software Developer/Feb'26/MPR-Feb'26.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\TH-PROJECT-NOTEBOOK\MPR\Role wise\Software Developer\Feb'26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F07AF6-7E6E-4B71-AF78-3605D9611998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E78BAEE-DDDB-4A60-841B-A5FDA7FBAD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="30">
   <si>
     <t>SR#</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>Switched to setup for Staging server provided by the Department for Hosting and security audit,                                  (1) Created and linked tables for audit and logging of different API requests being hit from different IP addresses</t>
+  </si>
+  <si>
+    <t>Compensatory leave due to office work on Sunday (08-02-26)</t>
   </si>
 </sst>
 </file>
@@ -171,7 +174,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -194,11 +197,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -218,32 +258,41 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -528,13 +577,13 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6" style="10" customWidth="1"/>
-    <col min="2" max="2" width="34" style="10" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" style="10" customWidth="1"/>
-    <col min="4" max="5" width="14.5703125" style="10" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.28515625" style="10" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="10"/>
+    <col min="1" max="1" width="6" style="9" customWidth="1"/>
+    <col min="2" max="2" width="34" style="9" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="9" customWidth="1"/>
+    <col min="4" max="5" width="14.5703125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.28515625" style="9" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -564,14 +613,14 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
     </row>
     <row r="3" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
@@ -600,14 +649,14 @@
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
     </row>
     <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
@@ -659,22 +708,22 @@
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="13">
         <v>46065</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -682,22 +731,22 @@
       <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="13">
         <v>46065</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -714,13 +763,13 @@
       <c r="D9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="13">
         <v>46065</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -728,22 +777,22 @@
       <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="13">
         <v>46065</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -751,22 +800,22 @@
       <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="13">
         <v>46065</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="15" t="s">
+      <c r="G11" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -774,22 +823,22 @@
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="13">
         <v>46064</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="G12" s="14" t="s">
         <v>21</v>
       </c>
     </row>
@@ -797,229 +846,230 @@
       <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="12"/>
+      <c r="G13" s="11"/>
     </row>
     <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
       <c r="F14" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="12"/>
-    </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="G14" s="11"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G15" s="12"/>
+      <c r="B15" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="18"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
     </row>
     <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="12"/>
+      <c r="G17" s="11"/>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="12"/>
+      <c r="G18" s="11"/>
     </row>
     <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G19" s="12"/>
+      <c r="G19" s="11"/>
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G20" s="12"/>
+      <c r="G20" s="11"/>
     </row>
     <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
       <c r="F21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G21" s="12"/>
+      <c r="G21" s="11"/>
     </row>
     <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="12"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
       <c r="F22" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G22" s="12"/>
+      <c r="G22" s="11"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
     </row>
     <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="12"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G24" s="12"/>
+      <c r="G24" s="11"/>
     </row>
     <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="12"/>
+      <c r="G25" s="11"/>
     </row>
     <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G26" s="12"/>
+      <c r="G26" s="11"/>
     </row>
     <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
       <c r="F27" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G27" s="12"/>
+      <c r="G27" s="11"/>
     </row>
     <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G28" s="12"/>
+      <c r="G28" s="11"/>
     </row>
     <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
       <c r="F29" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G29" s="12"/>
+      <c r="G29" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B15:G15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily MPR Update | 27-02-2026
</commit_message>
<xml_diff>
--- a/MPR/Role wise/Software Developer/Feb'26/MPR-Feb'26.xlsx
+++ b/MPR/Role wise/Software Developer/Feb'26/MPR-Feb'26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\TH-PROJECT-NOTEBOOK\MPR\Role wise\Software Developer\Feb'26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A420D20B-A507-4FFB-81B3-3672288EABD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3498A52F-4E85-4F0E-9350-6F0D3A3CC9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="54">
   <si>
     <t>SR#</t>
   </si>
@@ -72,12 +72,6 @@
     <t>On leave due to Family Emergency</t>
   </si>
   <si>
-    <t>Working on Reporting Section: (1) Headers - Geographical, Departments, Schemes and PLD wise</t>
-  </si>
-  <si>
-    <t>Working on Reporting Section: (1) Headers - Working on Scheme Code bug, Support bucket and Date filters.                (2) Body - Report table and Excel-Export Button</t>
-  </si>
-  <si>
     <t>Switched to setup for Staging server provided by the Department for Hosting and security audit,                                  (1) Migration of Test DB, with the exact collation and schema as the real one.</t>
   </si>
   <si>
@@ -123,21 +117,9 @@
     <t>Compensatory leave due to office work on Sunday (08-02-26)</t>
   </si>
   <si>
-    <t>Updation of Existing Enterprise / New Enterprise form fields in DB</t>
-  </si>
-  <si>
-    <t>Creation of DB Tables with linked constraints (Foreign keys with form type field - 'exep' for Existing Enterprise, 'newep' for New Enterprise</t>
-  </si>
-  <si>
     <t>CRUD (Create/Read/Update/Delete) APIS for Each Child Tables - Mandatory Fund, Licenses, Shop, and Segregated Media (Shop, Products and Enterprise Media)</t>
   </si>
   <si>
-    <t>Creation of UI/UX in React-Native, Dashboard screen with Analytics and CRP List with working filters.</t>
-  </si>
-  <si>
-    <t>Updation of CRP Filter API logic, adjustments and UI tweaks of Admin Dashboard as well as Fixing API permissions for IDOR</t>
-  </si>
-  <si>
     <t>Switched to setup CRP-EP App for Staging server,                                                   (1) Analysis of Suksham Udhyam Sakhi App,                                                                        (2) Enterprise forms and identification of fields currently leaking from API</t>
   </si>
   <si>
@@ -177,13 +159,43 @@
     <t>Creation of CRP-Panchayat rows with change button and delete icon with drop downs of districts, their subsequent blocks and their panchayats</t>
   </si>
   <si>
-    <t>Updation of old fields in form which were sending no data to API payload to now send data to correct API endpoint</t>
-  </si>
-  <si>
     <t>Migration of Test EPSMS DB Snapshot with schema and creation on staging server DB, created DB Indexes of related tables and merged with Django models in Backend</t>
   </si>
   <si>
     <t>Migration of Backend views, serializers and urls of EPSMS dev-backend to staging server and testing of APIS. Creation of Android package of Completed App ready for Round 1 Security Audit.</t>
+  </si>
+  <si>
+    <t>Received External Security Audit report of TMS, now working on fixing vulnerabilities</t>
+  </si>
+  <si>
+    <t>Switched to TMS on Staging server,    (1) Implementation of Server side Captacha and session validation               (2) Working on Business layer validations in Contact Person creation form.</t>
+  </si>
+  <si>
+    <t>Worked on Captcha implementation (frontend) in TMS based on vulnerabilities observed in Internal Audit report</t>
+  </si>
+  <si>
+    <t>Worked on IDOR error in TMS based on vulnerabilities observed in Internal Audit report</t>
+  </si>
+  <si>
+    <t>Creation of Developer's response of TMS based on vulnerabilities observed in Internal Audit report</t>
+  </si>
+  <si>
+    <t>Creation and planning of Client Requirements report based on security parameters and other limiting factors(Otp gateway, etc.)</t>
+  </si>
+  <si>
+    <t>Switched to LDMS,                               Working on Reporting Section: (1) Headers - Geographical, Departments, Schemes and PLD wise</t>
+  </si>
+  <si>
+    <t>Switched to LDMS,                               Working on Reporting Section: (1) Headers - Working on Scheme Code bug, Support bucket and Date filters.                (2) Body - Report table and Excel-Export Button</t>
+  </si>
+  <si>
+    <t>Switched to TMS on Staging server,    (1) Worked on configuring Pragma X-HTTP Headers                                             (2) Worked on Audit tables and optimizing cache services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switched to LDMS,                                           (1) Worked on Support Mapping Form and its APIs                                                    (2) Worked on created_by field not registering in child tables of form               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switched to LDMS,                                           (1) Worked on creation of Lucknow's Map for dashboard.                                                    (2) Worked on optimizing cache of LDMS API response               </t>
   </si>
 </sst>
 </file>
@@ -298,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -326,9 +338,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -670,21 +679,21 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-    </row>
-    <row r="3" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>7</v>
@@ -699,28 +708,28 @@
         <v>9</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-    </row>
-    <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+    </row>
+    <row r="5" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>7</v>
@@ -735,7 +744,7 @@
         <v>9</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="90" x14ac:dyDescent="0.25">
@@ -743,13 +752,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E6" s="5">
         <v>46065</v>
@@ -758,7 +767,7 @@
         <v>9</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="105" x14ac:dyDescent="0.25">
@@ -766,22 +775,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="12">
+      <c r="D7" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="11">
         <v>46065</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="13" t="s">
-        <v>22</v>
+      <c r="G7" s="12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="90" x14ac:dyDescent="0.25">
@@ -789,22 +798,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="12">
+        <v>21</v>
+      </c>
+      <c r="E8" s="11">
         <v>46065</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="13" t="s">
-        <v>22</v>
+      <c r="G8" s="12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="90" x14ac:dyDescent="0.25">
@@ -812,22 +821,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="12">
+        <v>21</v>
+      </c>
+      <c r="E9" s="11">
         <v>46065</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>22</v>
+      <c r="G9" s="12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="120" x14ac:dyDescent="0.25">
@@ -835,22 +844,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="12">
+        <v>21</v>
+      </c>
+      <c r="E10" s="11">
         <v>46065</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>22</v>
+      <c r="G10" s="12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="105" x14ac:dyDescent="0.25">
@@ -858,22 +867,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="12">
+        <v>21</v>
+      </c>
+      <c r="E11" s="11">
         <v>46065</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="13" t="s">
-        <v>22</v>
+      <c r="G11" s="12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="105" x14ac:dyDescent="0.25">
@@ -881,22 +890,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="11">
+        <v>46064</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>18</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="12">
-        <v>46064</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="120" x14ac:dyDescent="0.25">
@@ -904,22 +913,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="12">
+      <c r="D13" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="11">
         <v>46069</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="13" t="s">
-        <v>29</v>
+      <c r="G13" s="12" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -927,298 +936,338 @@
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="12">
+      <c r="D14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="11">
         <v>46069</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="13" t="s">
-        <v>30</v>
+      <c r="G14" s="12" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17"/>
+      <c r="B15" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
     </row>
     <row r="17" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>37</v>
+      <c r="B17" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="12">
+        <v>16</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="11">
         <v>46069</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="13" t="s">
-        <v>31</v>
+      <c r="G17" s="12" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="13" t="s">
-        <v>38</v>
+      <c r="B18" s="12" t="s">
+        <v>32</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="12">
+      <c r="D18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="11">
         <v>46073</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="13" t="s">
-        <v>32</v>
+      <c r="G18" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="13" t="s">
-        <v>39</v>
+      <c r="B19" s="12" t="s">
+        <v>33</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="12">
+      <c r="D19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="11">
         <v>46073</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G19" s="13" t="s">
-        <v>33</v>
+      <c r="G19" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>44</v>
+      <c r="B20" s="12" t="s">
+        <v>38</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="12">
+      <c r="D20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="11">
         <v>46073</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G20" s="13" t="s">
-        <v>45</v>
+      <c r="G20" s="12" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="13" t="s">
-        <v>41</v>
+      <c r="B21" s="12" t="s">
+        <v>35</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="12">
+        <v>16</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" s="11">
         <v>46073</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G21" s="13" t="s">
-        <v>46</v>
+      <c r="G21" s="12" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="13" t="s">
-        <v>40</v>
+      <c r="B22" s="12" t="s">
+        <v>34</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="12">
+      <c r="D22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="11">
         <v>46077</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G22" s="13" t="s">
-        <v>47</v>
+      <c r="G22" s="12" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
     </row>
     <row r="24" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="13" t="s">
-        <v>42</v>
+      <c r="B24" s="12" t="s">
+        <v>36</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24" s="12">
+      <c r="D24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="11">
         <v>46077</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G24" s="13" t="s">
-        <v>48</v>
+      <c r="G24" s="12" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
-      <c r="B25" s="13" t="s">
-        <v>43</v>
+      <c r="B25" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25" s="12">
+        <v>16</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="11">
         <v>46077</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="G25" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
+      <c r="B26" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" s="11">
+        <v>46079</v>
+      </c>
       <c r="F26" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G26" s="10"/>
-    </row>
-    <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="G26" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
+      <c r="B27" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" s="11">
+        <v>46079</v>
+      </c>
       <c r="F27" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G27" s="10"/>
-    </row>
-    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="G27" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="10"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
+      <c r="B28" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="11">
+        <v>46081</v>
+      </c>
       <c r="F28" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G28" s="10"/>
-    </row>
-    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="G28" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
+      <c r="B29" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="11">
+        <v>46090</v>
+      </c>
       <c r="F29" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G29" s="10"/>
+      <c r="G29" s="12" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>